<commit_message>
fix: resolve WebKit cross-browser test failures
</commit_message>
<xml_diff>
--- a/docs/test-analiz-dokumani.xlsx
+++ b/docs/test-analiz-dokumani.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="127">
   <si>
     <t>Modül</t>
   </si>
@@ -144,68 +144,6 @@
     <t>#result alanı 'workspace' metnini içerir</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t xml:space="preserve">Chromium: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1B7F3A"/>
-        <sz val="13"/>
-      </rPr>
-      <t>✓</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t xml:space="preserve">
-Firefox: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1B7F3A"/>
-        <sz val="13"/>
-      </rPr>
-      <t>✓</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t xml:space="preserve">
-WebKit: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFB30000"/>
-        <sz val="13"/>
-      </rPr>
-      <t>✗</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve"> Test timeout of 30000ms exceeded.</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <color rgb="FF666666"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">
-(2026-05-26)</t>
-    </r>
-  </si>
-  <si>
     <t>TC-ELE-P-04</t>
   </si>
   <si>
@@ -238,68 +176,6 @@
   </si>
   <si>
     <t>Yeni satır tablonun en altında görünür ve eklenen değerleri içerir</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t xml:space="preserve">Chromium: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1B7F3A"/>
-        <sz val="13"/>
-      </rPr>
-      <t>✓</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t xml:space="preserve">
-Firefox: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1B7F3A"/>
-        <sz val="13"/>
-      </rPr>
-      <t>✓</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t xml:space="preserve">
-WebKit: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFB30000"/>
-        <sz val="13"/>
-      </rPr>
-      <t>✗</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve"> TimeoutError: locator.click: Timeout 10000ms exceeded.</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <color rgb="FF666666"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">
-(2026-05-26)</t>
-    </r>
   </si>
   <si>
     <t>TC-ELE-N-06</t>
@@ -332,68 +208,6 @@
   </si>
   <si>
     <t>3 farklı mesaj DOM'da görünür: #doubleClickMessage, #rightClickMessage, #dynamicClickMessage</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t xml:space="preserve">Chromium: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1B7F3A"/>
-        <sz val="13"/>
-      </rPr>
-      <t>✓</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t xml:space="preserve">
-Firefox: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF1B7F3A"/>
-        <sz val="13"/>
-      </rPr>
-      <t>✓</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t xml:space="preserve">
-WebKit: </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FFB30000"/>
-        <sz val="13"/>
-      </rPr>
-      <t>✗</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve"> TimeoutError: locator.dblclick: Timeout 10000ms exceeded.</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <color rgb="FF666666"/>
-        <sz val="9"/>
-      </rPr>
-      <t xml:space="preserve">
-(2026-05-26)</t>
-    </r>
   </si>
   <si>
     <t>TC-ELE-P-08</t>
@@ -686,7 +500,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -716,11 +530,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8D7DA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF5A4A4"/>
       </patternFill>
     </fill>
     <fill>
@@ -761,7 +570,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -790,13 +599,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1237,8 +1043,8 @@
       <c r="F4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G4" s="10" t="s">
-        <v>24</v>
+      <c r="G4" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1246,19 +1052,19 @@
         <v>7</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>29</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>13</v>
@@ -1269,22 +1075,22 @@
         <v>7</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>35</v>
+      <c r="G6" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1292,19 +1098,19 @@
         <v>7</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>37</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>39</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>13</v>
@@ -1315,22 +1121,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>45</v>
+      <c r="G8" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1338,19 +1144,19 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>47</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>50</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>13</v>
@@ -1361,19 +1167,19 @@
         <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="F10" s="9" t="s">
         <v>52</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>55</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>13</v>
@@ -1384,364 +1190,364 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="G11" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="C12" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="D12" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="G12" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="C13" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="D13" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="G12" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="F13" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="6" t="s">
+      <c r="E14" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="F14" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="F14" s="9" t="s">
+      <c r="E15" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G14" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="F15" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="F15" s="9" t="s">
+      <c r="E16" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="G15" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="F16" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="F16" s="6" t="s">
+      <c r="E17" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="G16" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B17" s="8" t="s">
+      <c r="F17" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="G17" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E17" s="9" t="s">
+      <c r="B18" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="C18" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="G17" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="D18" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="E18" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="G18" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="C19" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="D19" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="G18" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B19" s="5" t="s">
+      <c r="F19" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="G19" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="E19" s="6" t="s">
+      <c r="C20" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="D20" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B20" s="5" t="s">
+      <c r="E20" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="F20" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="G20" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="D21" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="G20" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B21" s="5" t="s">
+      <c r="E21" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="G21" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="C22" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="D22" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G21" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B22" s="8" t="s">
+      <c r="F22" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="G22" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="E22" s="9" t="s">
+      <c r="C23" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="D23" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="G22" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B23" s="5" t="s">
+      <c r="E23" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="G23" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="C24" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="D24" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E24" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="G23" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B24" s="8" t="s">
+      <c r="F24" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="G24" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="E24" s="9" t="s">
+      <c r="C25" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="D25" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="G24" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B25" s="5" t="s">
+      <c r="E25" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="G25" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B26" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="C26" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="D26" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="G25" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" ht="60" customHeight="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B26" s="5" t="s">
+      <c r="E26" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>126</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="G26" s="7" t="s">
         <v>13</v>

</xml_diff>